<commit_message>
parse timesheet excel by AI
</commit_message>
<xml_diff>
--- a/sample_data/TMV_Timesheet_March_2026.xlsx
+++ b/sample_data/TMV_Timesheet_March_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/snarayanaswamy/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0ACC26A-7C6E-F443-9B71-D78838414DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18AFDBD-7576-F945-B4BA-09AE782B6033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="69">
   <si>
     <t>Project Name: TMV Holding</t>
   </si>
@@ -241,6 +241,9 @@
   </si>
   <si>
     <t>cost</t>
+  </si>
+  <si>
+    <t>Cosst</t>
   </si>
 </sst>
 </file>
@@ -1230,7 +1233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="181">
+  <cellXfs count="177">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1493,69 +1496,141 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="7" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="7" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="7" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="15" fontId="3" fillId="7" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="15" fontId="3" fillId="7" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1579,142 +1654,60 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="15" fontId="3" fillId="7" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="15" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="7" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="7" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="15" fontId="3" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="7" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1977,20 +1970,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="122">
+      <c r="A1" s="150">
         <v>46082</v>
       </c>
-      <c r="B1" s="123"/>
-      <c r="C1" s="123"/>
-      <c r="D1" s="123"/>
-      <c r="E1" s="123"/>
-      <c r="F1" s="123"/>
-      <c r="G1" s="123"/>
-      <c r="H1" s="123"/>
-      <c r="I1" s="123"/>
-      <c r="J1" s="123"/>
-      <c r="K1" s="123"/>
-      <c r="L1" s="124"/>
+      <c r="B1" s="151"/>
+      <c r="C1" s="151"/>
+      <c r="D1" s="151"/>
+      <c r="E1" s="151"/>
+      <c r="F1" s="151"/>
+      <c r="G1" s="151"/>
+      <c r="H1" s="151"/>
+      <c r="I1" s="151"/>
+      <c r="J1" s="151"/>
+      <c r="K1" s="151"/>
+      <c r="L1" s="152"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
@@ -2006,20 +1999,20 @@
     <row r="2" spans="1:31" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="29"/>
       <c r="B2" s="29"/>
-      <c r="C2" s="125" t="s">
+      <c r="C2" s="153" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="126"/>
-      <c r="E2" s="125" t="s">
+      <c r="D2" s="154"/>
+      <c r="E2" s="153" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="128"/>
-      <c r="G2" s="128"/>
-      <c r="H2" s="128"/>
-      <c r="I2" s="128"/>
-      <c r="J2" s="128"/>
-      <c r="K2" s="128"/>
-      <c r="L2" s="126"/>
+      <c r="F2" s="158"/>
+      <c r="G2" s="158"/>
+      <c r="H2" s="158"/>
+      <c r="I2" s="158"/>
+      <c r="J2" s="158"/>
+      <c r="K2" s="158"/>
+      <c r="L2" s="154"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
@@ -2030,83 +2023,87 @@
       <c r="AD2" s="1"/>
     </row>
     <row r="3" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="117" t="s">
+      <c r="A3" s="155" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="117" t="s">
+      <c r="B3" s="155" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="117" t="s">
+      <c r="C3" s="155" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="105"/>
-      <c r="E3" s="117" t="s">
+      <c r="D3" s="134"/>
+      <c r="E3" s="155" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="105"/>
-      <c r="G3" s="127" t="s">
+      <c r="F3" s="134"/>
+      <c r="G3" s="156" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="107"/>
-      <c r="I3" s="117" t="s">
+      <c r="H3" s="157"/>
+      <c r="I3" s="155" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="117" t="s">
-        <v>8</v>
-      </c>
-      <c r="K3" s="118" t="s">
+      <c r="J3" s="155" t="s">
+        <v>8</v>
+      </c>
+      <c r="K3" s="167" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="117" t="s">
+      <c r="L3" s="155" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="167" t="s">
+      <c r="M3" s="169" t="s">
         <v>11</v>
       </c>
-      <c r="N3" s="176"/>
-      <c r="O3" s="176"/>
-      <c r="P3" s="173" t="s">
+      <c r="N3" s="155" t="s">
+        <v>66</v>
+      </c>
+      <c r="O3" s="169" t="s">
+        <v>68</v>
+      </c>
+      <c r="P3" s="159" t="s">
         <v>12</v>
       </c>
-      <c r="Q3" s="109"/>
-      <c r="R3" s="109"/>
-      <c r="S3" s="109"/>
-      <c r="T3" s="109"/>
-      <c r="U3" s="110"/>
-      <c r="W3" s="116" t="s">
+      <c r="Q3" s="160"/>
+      <c r="R3" s="160"/>
+      <c r="S3" s="160"/>
+      <c r="T3" s="160"/>
+      <c r="U3" s="161"/>
+      <c r="W3" s="165" t="s">
         <v>13</v>
       </c>
-      <c r="X3" s="109"/>
-      <c r="Y3" s="110"/>
+      <c r="X3" s="160"/>
+      <c r="Y3" s="161"/>
       <c r="AB3" s="1"/>
       <c r="AC3" s="1"/>
     </row>
     <row r="4" spans="1:31" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="105"/>
-      <c r="B4" s="105"/>
-      <c r="C4" s="105"/>
-      <c r="D4" s="105"/>
-      <c r="E4" s="105"/>
-      <c r="F4" s="105"/>
-      <c r="G4" s="107"/>
-      <c r="H4" s="107"/>
-      <c r="I4" s="105"/>
-      <c r="J4" s="105"/>
-      <c r="K4" s="119"/>
-      <c r="L4" s="105"/>
-      <c r="M4" s="168"/>
-      <c r="N4" s="177" t="s">
+      <c r="A4" s="134"/>
+      <c r="B4" s="134"/>
+      <c r="C4" s="134"/>
+      <c r="D4" s="134"/>
+      <c r="E4" s="134"/>
+      <c r="F4" s="134"/>
+      <c r="G4" s="157"/>
+      <c r="H4" s="157"/>
+      <c r="I4" s="134"/>
+      <c r="J4" s="134"/>
+      <c r="K4" s="168"/>
+      <c r="L4" s="134"/>
+      <c r="M4" s="170"/>
+      <c r="N4" s="134" t="s">
         <v>66</v>
       </c>
-      <c r="O4" s="177" t="s">
+      <c r="O4" s="170" t="s">
         <v>67</v>
       </c>
-      <c r="P4" s="99" t="s">
+      <c r="P4" s="166" t="s">
         <v>14</v>
       </c>
-      <c r="Q4" s="100"/>
-      <c r="R4" s="100"/>
-      <c r="S4" s="101"/>
+      <c r="Q4" s="162"/>
+      <c r="R4" s="162"/>
+      <c r="S4" s="163"/>
       <c r="T4" s="39" t="s">
         <v>15</v>
       </c>
@@ -2133,18 +2130,18 @@
       <c r="B5" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="102" t="s">
+      <c r="C5" s="130" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="103"/>
-      <c r="E5" s="104" t="s">
+      <c r="D5" s="105"/>
+      <c r="E5" s="135" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="105"/>
-      <c r="G5" s="106">
+      <c r="F5" s="134"/>
+      <c r="G5" s="173">
         <v>45873</v>
       </c>
-      <c r="H5" s="107"/>
+      <c r="H5" s="157"/>
       <c r="I5" s="33">
         <f t="shared" ref="I5:I14" si="0">$U$13</f>
         <v>176</v>
@@ -2161,19 +2158,19 @@
         <f>IF(I5=K5,"",(I5-K5)/8)</f>
         <v>1</v>
       </c>
-      <c r="M5" s="169"/>
-      <c r="N5" s="178">
+      <c r="M5" s="94"/>
+      <c r="N5" s="98">
         <v>100</v>
       </c>
-      <c r="O5" s="178">
+      <c r="O5" s="98">
         <v>20</v>
       </c>
-      <c r="P5" s="97" t="s">
+      <c r="P5" s="146" t="s">
         <v>23</v>
       </c>
-      <c r="Q5" s="100"/>
-      <c r="R5" s="100"/>
-      <c r="S5" s="101"/>
+      <c r="Q5" s="162"/>
+      <c r="R5" s="162"/>
+      <c r="S5" s="163"/>
       <c r="T5" s="9">
         <v>10</v>
       </c>
@@ -2199,18 +2196,18 @@
       <c r="B6" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="108" t="s">
+      <c r="C6" s="113" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="103"/>
-      <c r="E6" s="104" t="s">
+      <c r="D6" s="105"/>
+      <c r="E6" s="135" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="105"/>
-      <c r="G6" s="106">
+      <c r="F6" s="134"/>
+      <c r="G6" s="173">
         <v>45873</v>
       </c>
-      <c r="H6" s="107"/>
+      <c r="H6" s="157"/>
       <c r="I6" s="33">
         <f t="shared" si="0"/>
         <v>176</v>
@@ -2230,18 +2227,18 @@
       <c r="M6" s="91">
         <v>46106</v>
       </c>
-      <c r="N6" s="178">
+      <c r="N6" s="98">
         <v>89</v>
       </c>
-      <c r="O6" s="178">
+      <c r="O6" s="98">
         <v>30</v>
       </c>
-      <c r="P6" s="174" t="s">
+      <c r="P6" s="175" t="s">
         <v>29</v>
       </c>
-      <c r="Q6" s="100"/>
-      <c r="R6" s="100"/>
-      <c r="S6" s="101"/>
+      <c r="Q6" s="162"/>
+      <c r="R6" s="162"/>
+      <c r="S6" s="163"/>
       <c r="T6" s="9">
         <v>0</v>
       </c>
@@ -2261,18 +2258,18 @@
       <c r="B7" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="112" t="s">
+      <c r="C7" s="106" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="103"/>
-      <c r="E7" s="113" t="s">
+      <c r="D7" s="105"/>
+      <c r="E7" s="144" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="114"/>
-      <c r="G7" s="106">
+      <c r="F7" s="145"/>
+      <c r="G7" s="173">
         <v>45877</v>
       </c>
-      <c r="H7" s="107"/>
+      <c r="H7" s="157"/>
       <c r="I7" s="33">
         <f t="shared" si="0"/>
         <v>176</v>
@@ -2289,19 +2286,19 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="M7" s="169"/>
-      <c r="N7" s="178">
+      <c r="M7" s="94"/>
+      <c r="N7" s="98">
         <v>90</v>
       </c>
-      <c r="O7" s="178">
+      <c r="O7" s="98">
         <v>70</v>
       </c>
-      <c r="P7" s="111" t="s">
+      <c r="P7" s="176" t="s">
         <v>33</v>
       </c>
-      <c r="Q7" s="95"/>
-      <c r="R7" s="95"/>
-      <c r="S7" s="96"/>
+      <c r="Q7" s="172"/>
+      <c r="R7" s="172"/>
+      <c r="S7" s="119"/>
       <c r="T7" s="14">
         <f t="shared" ref="T7:U7" si="4">T5-T6</f>
         <v>10</v>
@@ -2322,18 +2319,18 @@
       <c r="B8" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="112" t="s">
+      <c r="C8" s="106" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="103"/>
-      <c r="E8" s="113" t="s">
+      <c r="D8" s="105"/>
+      <c r="E8" s="144" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="114"/>
-      <c r="G8" s="115">
+      <c r="F8" s="145"/>
+      <c r="G8" s="164">
         <v>45890</v>
       </c>
-      <c r="H8" s="107"/>
+      <c r="H8" s="157"/>
       <c r="I8" s="33">
         <f t="shared" si="0"/>
         <v>176</v>
@@ -2350,21 +2347,21 @@
         <f t="shared" ref="L8" si="6">IF(I8=K8,"",(I8-K8)/8)</f>
         <v/>
       </c>
-      <c r="M8" s="169"/>
-      <c r="N8" s="178">
+      <c r="M8" s="94"/>
+      <c r="N8" s="98">
         <v>38</v>
       </c>
-      <c r="O8" s="178">
+      <c r="O8" s="98">
         <v>90</v>
       </c>
-      <c r="P8" s="175" t="s">
+      <c r="P8" s="174" t="s">
         <v>36</v>
       </c>
-      <c r="Q8" s="109"/>
-      <c r="R8" s="109"/>
-      <c r="S8" s="109"/>
-      <c r="T8" s="109"/>
-      <c r="U8" s="110"/>
+      <c r="Q8" s="160"/>
+      <c r="R8" s="160"/>
+      <c r="S8" s="160"/>
+      <c r="T8" s="160"/>
+      <c r="U8" s="161"/>
       <c r="V8" s="1"/>
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
@@ -2377,18 +2374,18 @@
       <c r="B9" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="112" t="s">
+      <c r="C9" s="106" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="103"/>
-      <c r="E9" s="113" t="s">
+      <c r="D9" s="105"/>
+      <c r="E9" s="144" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="114"/>
-      <c r="G9" s="120">
+      <c r="F9" s="145"/>
+      <c r="G9" s="148">
         <v>45978</v>
       </c>
-      <c r="H9" s="121"/>
+      <c r="H9" s="149"/>
       <c r="I9" s="33">
         <f t="shared" si="0"/>
         <v>176</v>
@@ -2405,19 +2402,19 @@
         <f>IF(I9=K9,"",(I9-K9)/8)</f>
         <v>1</v>
       </c>
-      <c r="M9" s="170"/>
-      <c r="N9" s="178">
+      <c r="M9" s="95"/>
+      <c r="N9" s="98">
         <v>89</v>
       </c>
-      <c r="O9" s="178">
+      <c r="O9" s="98">
         <v>20</v>
       </c>
-      <c r="P9" s="99" t="s">
+      <c r="P9" s="166" t="s">
         <v>14</v>
       </c>
-      <c r="Q9" s="100"/>
-      <c r="R9" s="100"/>
-      <c r="S9" s="101"/>
+      <c r="Q9" s="162"/>
+      <c r="R9" s="162"/>
+      <c r="S9" s="163"/>
       <c r="T9" s="39" t="s">
         <v>15</v>
       </c>
@@ -2436,18 +2433,18 @@
       <c r="B10" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="112" t="s">
+      <c r="C10" s="106" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="103"/>
-      <c r="E10" s="113" t="s">
+      <c r="D10" s="105"/>
+      <c r="E10" s="144" t="s">
         <v>42</v>
       </c>
-      <c r="F10" s="114"/>
-      <c r="G10" s="120">
+      <c r="F10" s="145"/>
+      <c r="G10" s="148">
         <v>45962</v>
       </c>
-      <c r="H10" s="121"/>
+      <c r="H10" s="149"/>
       <c r="I10" s="33">
         <f t="shared" si="0"/>
         <v>176</v>
@@ -2464,19 +2461,19 @@
         <f>IF(I10=K10,"",(I10-K10)/8)</f>
         <v>2</v>
       </c>
-      <c r="M10" s="169"/>
-      <c r="N10" s="178">
+      <c r="M10" s="94"/>
+      <c r="N10" s="98">
         <v>47</v>
       </c>
-      <c r="O10" s="178">
+      <c r="O10" s="98">
         <v>60</v>
       </c>
-      <c r="P10" s="97" t="s">
+      <c r="P10" s="146" t="s">
         <v>23</v>
       </c>
-      <c r="Q10" s="97"/>
-      <c r="R10" s="97"/>
-      <c r="S10" s="98"/>
+      <c r="Q10" s="146"/>
+      <c r="R10" s="146"/>
+      <c r="S10" s="147"/>
       <c r="T10" s="9">
         <v>12</v>
       </c>
@@ -2496,18 +2493,18 @@
       <c r="B11" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="108" t="s">
+      <c r="C11" s="113" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="105"/>
-      <c r="E11" s="104" t="s">
+      <c r="D11" s="134"/>
+      <c r="E11" s="135" t="s">
         <v>45</v>
       </c>
-      <c r="F11" s="105"/>
-      <c r="G11" s="139">
+      <c r="F11" s="134"/>
+      <c r="G11" s="136">
         <v>46009</v>
       </c>
-      <c r="H11" s="105"/>
+      <c r="H11" s="134"/>
       <c r="I11" s="33">
         <f t="shared" si="0"/>
         <v>176</v>
@@ -2524,19 +2521,19 @@
         <f>IF(I11=K11,"",(I11-K11)/8)</f>
         <v>4</v>
       </c>
-      <c r="M11" s="169"/>
-      <c r="N11" s="178">
+      <c r="M11" s="94"/>
+      <c r="N11" s="98">
         <v>89</v>
       </c>
-      <c r="O11" s="178">
+      <c r="O11" s="98">
         <v>70</v>
       </c>
-      <c r="P11" s="97" t="s">
+      <c r="P11" s="146" t="s">
         <v>29</v>
       </c>
-      <c r="Q11" s="97"/>
-      <c r="R11" s="97"/>
-      <c r="S11" s="98"/>
+      <c r="Q11" s="146"/>
+      <c r="R11" s="146"/>
+      <c r="S11" s="147"/>
       <c r="T11" s="16">
         <v>0</v>
       </c>
@@ -2556,18 +2553,18 @@
       <c r="B12" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="108" t="s">
+      <c r="C12" s="113" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="105"/>
-      <c r="E12" s="104" t="s">
+      <c r="D12" s="134"/>
+      <c r="E12" s="135" t="s">
         <v>45</v>
       </c>
-      <c r="F12" s="105"/>
-      <c r="G12" s="140">
+      <c r="F12" s="134"/>
+      <c r="G12" s="138">
         <v>46050</v>
       </c>
-      <c r="H12" s="141"/>
+      <c r="H12" s="139"/>
       <c r="I12" s="33">
         <f t="shared" si="0"/>
         <v>176</v>
@@ -2584,19 +2581,19 @@
         <f>IF(I12=K12,"",(I12-K12)/8)</f>
         <v>1</v>
       </c>
-      <c r="M12" s="171"/>
-      <c r="N12" s="178">
+      <c r="M12" s="96"/>
+      <c r="N12" s="98">
         <v>70</v>
       </c>
-      <c r="O12" s="178">
+      <c r="O12" s="98">
         <v>90</v>
       </c>
-      <c r="P12" s="94" t="s">
+      <c r="P12" s="171" t="s">
         <v>33</v>
       </c>
-      <c r="Q12" s="95"/>
-      <c r="R12" s="95"/>
-      <c r="S12" s="96"/>
+      <c r="Q12" s="172"/>
+      <c r="R12" s="172"/>
+      <c r="S12" s="119"/>
       <c r="T12" s="14">
         <f>T10-T11</f>
         <v>12</v>
@@ -2616,18 +2613,18 @@
       <c r="B13" s="79" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="142" t="s">
+      <c r="C13" s="140" t="s">
         <v>49</v>
       </c>
-      <c r="D13" s="143"/>
-      <c r="E13" s="104" t="s">
+      <c r="D13" s="141"/>
+      <c r="E13" s="135" t="s">
         <v>50</v>
       </c>
-      <c r="F13" s="105"/>
-      <c r="G13" s="140">
+      <c r="F13" s="134"/>
+      <c r="G13" s="138">
         <v>46059</v>
       </c>
-      <c r="H13" s="141"/>
+      <c r="H13" s="139"/>
       <c r="I13" s="33">
         <f t="shared" si="0"/>
         <v>176</v>
@@ -2643,19 +2640,19 @@
       <c r="L13" s="82">
         <v>1</v>
       </c>
-      <c r="M13" s="169"/>
-      <c r="N13" s="179">
+      <c r="M13" s="94"/>
+      <c r="N13" s="98">
         <v>50</v>
       </c>
-      <c r="O13" s="179">
+      <c r="O13" s="98">
         <v>20</v>
       </c>
-      <c r="P13" s="144" t="s">
+      <c r="P13" s="126" t="s">
         <v>51</v>
       </c>
-      <c r="Q13" s="144"/>
-      <c r="R13" s="144"/>
-      <c r="S13" s="145"/>
+      <c r="Q13" s="126"/>
+      <c r="R13" s="126"/>
+      <c r="S13" s="127"/>
       <c r="T13" s="41">
         <f>T7+T12</f>
         <v>22</v>
@@ -2675,18 +2672,18 @@
       <c r="B14" s="79" t="s">
         <v>52</v>
       </c>
-      <c r="C14" s="142" t="s">
+      <c r="C14" s="140" t="s">
         <v>53</v>
       </c>
-      <c r="D14" s="143"/>
-      <c r="E14" s="104" t="s">
+      <c r="D14" s="141"/>
+      <c r="E14" s="135" t="s">
         <v>54</v>
       </c>
-      <c r="F14" s="105"/>
-      <c r="G14" s="140">
+      <c r="F14" s="134"/>
+      <c r="G14" s="138">
         <v>46099</v>
       </c>
-      <c r="H14" s="141"/>
+      <c r="H14" s="139"/>
       <c r="I14" s="33">
         <f t="shared" si="0"/>
         <v>176</v>
@@ -2702,11 +2699,11 @@
       <c r="L14" s="82">
         <v>0</v>
       </c>
-      <c r="M14" s="169"/>
-      <c r="N14" s="179">
+      <c r="M14" s="94"/>
+      <c r="N14" s="98">
         <v>80</v>
       </c>
-      <c r="O14" s="179">
+      <c r="O14" s="98">
         <v>60</v>
       </c>
       <c r="P14" s="71"/>
@@ -2723,9 +2720,9 @@
       <c r="A15" s="80">
         <v>11</v>
       </c>
-      <c r="M15" s="170"/>
-      <c r="N15" s="178"/>
-      <c r="O15" s="178"/>
+      <c r="M15" s="95"/>
+      <c r="N15" s="98"/>
+      <c r="O15" s="98"/>
       <c r="P15" s="71"/>
       <c r="Q15" s="71"/>
       <c r="R15" s="71"/>
@@ -2739,12 +2736,12 @@
     <row r="16" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="34"/>
       <c r="B16" s="81"/>
-      <c r="C16" s="131"/>
-      <c r="D16" s="105"/>
-      <c r="E16" s="131"/>
-      <c r="F16" s="105"/>
-      <c r="G16" s="146"/>
-      <c r="H16" s="147"/>
+      <c r="C16" s="137"/>
+      <c r="D16" s="134"/>
+      <c r="E16" s="137"/>
+      <c r="F16" s="134"/>
+      <c r="G16" s="128"/>
+      <c r="H16" s="129"/>
       <c r="I16" s="44">
         <f>SUM(I5:I12)</f>
         <v>1408</v>
@@ -2761,9 +2758,9 @@
         <f>SUM(L5:L12)</f>
         <v>14</v>
       </c>
-      <c r="M16" s="172"/>
-      <c r="N16" s="180"/>
-      <c r="O16" s="180"/>
+      <c r="M16" s="97"/>
+      <c r="N16" s="99"/>
+      <c r="O16" s="99"/>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
       <c r="X16" s="1"/>
@@ -2788,8 +2785,8 @@
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
-      <c r="N17" s="166"/>
-      <c r="O17" s="166"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
       <c r="R17" s="1"/>
@@ -2804,57 +2801,57 @@
     </row>
     <row r="18" spans="1:31" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="30"/>
-      <c r="B18" s="148" t="s">
+      <c r="B18" s="131" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="149"/>
-      <c r="D18" s="149"/>
-      <c r="E18" s="149"/>
-      <c r="F18" s="149"/>
-      <c r="G18" s="149"/>
-      <c r="H18" s="149"/>
-      <c r="I18" s="149"/>
-      <c r="J18" s="149"/>
-      <c r="K18" s="149"/>
-      <c r="L18" s="149"/>
-      <c r="M18" s="149"/>
-      <c r="N18" s="149"/>
-      <c r="O18" s="149"/>
-      <c r="P18" s="149"/>
-      <c r="Q18" s="149"/>
-      <c r="R18" s="149"/>
-      <c r="S18" s="149"/>
-      <c r="T18" s="149"/>
-      <c r="U18" s="149"/>
-      <c r="V18" s="149"/>
-      <c r="W18" s="149"/>
-      <c r="X18" s="149"/>
-      <c r="Y18" s="149"/>
-      <c r="Z18" s="149"/>
-      <c r="AA18" s="149"/>
-      <c r="AB18" s="150"/>
+      <c r="C18" s="132"/>
+      <c r="D18" s="132"/>
+      <c r="E18" s="132"/>
+      <c r="F18" s="132"/>
+      <c r="G18" s="132"/>
+      <c r="H18" s="132"/>
+      <c r="I18" s="132"/>
+      <c r="J18" s="132"/>
+      <c r="K18" s="132"/>
+      <c r="L18" s="132"/>
+      <c r="M18" s="132"/>
+      <c r="N18" s="132"/>
+      <c r="O18" s="132"/>
+      <c r="P18" s="132"/>
+      <c r="Q18" s="132"/>
+      <c r="R18" s="132"/>
+      <c r="S18" s="132"/>
+      <c r="T18" s="132"/>
+      <c r="U18" s="132"/>
+      <c r="V18" s="132"/>
+      <c r="W18" s="132"/>
+      <c r="X18" s="132"/>
+      <c r="Y18" s="132"/>
+      <c r="Z18" s="132"/>
+      <c r="AA18" s="132"/>
+      <c r="AB18" s="133"/>
       <c r="AC18" s="18"/>
       <c r="AD18" s="18"/>
       <c r="AE18" s="1"/>
     </row>
     <row r="19" spans="1:31" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="43"/>
-      <c r="B19" s="154" t="s">
+      <c r="B19" s="107" t="s">
         <v>2</v>
       </c>
-      <c r="C19" s="156" t="s">
+      <c r="C19" s="109" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="157"/>
-      <c r="E19" s="134" t="s">
+      <c r="D19" s="110"/>
+      <c r="E19" s="122" t="s">
         <v>55</v>
       </c>
-      <c r="F19" s="136" t="s">
+      <c r="F19" s="124" t="s">
         <v>16</v>
       </c>
-      <c r="G19" s="137"/>
-      <c r="H19" s="137"/>
-      <c r="I19" s="138"/>
+      <c r="G19" s="125"/>
+      <c r="H19" s="125"/>
+      <c r="I19" s="112"/>
       <c r="J19" s="45">
         <f>A1</f>
         <v>46082</v>
@@ -2925,10 +2922,10 @@
     </row>
     <row r="20" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="43"/>
-      <c r="B20" s="155"/>
-      <c r="C20" s="158"/>
-      <c r="D20" s="138"/>
-      <c r="E20" s="135"/>
+      <c r="B20" s="108"/>
+      <c r="C20" s="111"/>
+      <c r="D20" s="112"/>
+      <c r="E20" s="123"/>
       <c r="F20" s="39" t="s">
         <v>56</v>
       </c>
@@ -3014,10 +3011,10 @@
       <c r="B21" s="8">
         <v>1</v>
       </c>
-      <c r="C21" s="102" t="s">
+      <c r="C21" s="130" t="s">
         <v>21</v>
       </c>
-      <c r="D21" s="103"/>
+      <c r="D21" s="105"/>
       <c r="E21" s="21" t="s">
         <v>60</v>
       </c>
@@ -3084,10 +3081,10 @@
       <c r="B22" s="8">
         <v>2</v>
       </c>
-      <c r="C22" s="108" t="s">
+      <c r="C22" s="113" t="s">
         <v>27</v>
       </c>
-      <c r="D22" s="103"/>
+      <c r="D22" s="105"/>
       <c r="E22" s="21" t="s">
         <v>61</v>
       </c>
@@ -3154,10 +3151,10 @@
       <c r="B23" s="8">
         <v>3</v>
       </c>
-      <c r="C23" s="112" t="s">
+      <c r="C23" s="106" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="103"/>
+      <c r="D23" s="105"/>
       <c r="E23" s="21" t="s">
         <v>62</v>
       </c>
@@ -3224,10 +3221,10 @@
       <c r="B24" s="8">
         <v>5</v>
       </c>
-      <c r="C24" s="112" t="s">
+      <c r="C24" s="106" t="s">
         <v>35</v>
       </c>
-      <c r="D24" s="103"/>
+      <c r="D24" s="105"/>
       <c r="E24" s="21" t="s">
         <v>63</v>
       </c>
@@ -3294,10 +3291,10 @@
       <c r="B25" s="64">
         <v>6</v>
       </c>
-      <c r="C25" s="112" t="s">
+      <c r="C25" s="106" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="103"/>
+      <c r="D25" s="105"/>
       <c r="E25" s="65" t="s">
         <v>64</v>
       </c>
@@ -3364,10 +3361,10 @@
       <c r="B26" s="64">
         <v>7</v>
       </c>
-      <c r="C26" s="112" t="s">
+      <c r="C26" s="106" t="s">
         <v>41</v>
       </c>
-      <c r="D26" s="103"/>
+      <c r="D26" s="105"/>
       <c r="E26" s="65" t="s">
         <v>42</v>
       </c>
@@ -3434,10 +3431,10 @@
       <c r="B27" s="64">
         <v>9</v>
       </c>
-      <c r="C27" s="112" t="s">
+      <c r="C27" s="106" t="s">
         <v>44</v>
       </c>
-      <c r="D27" s="103"/>
+      <c r="D27" s="105"/>
       <c r="E27" s="65" t="s">
         <v>28</v>
       </c>
@@ -3504,10 +3501,10 @@
       <c r="B28" s="64">
         <v>10</v>
       </c>
-      <c r="C28" s="132" t="s">
+      <c r="C28" s="100" t="s">
         <v>47</v>
       </c>
-      <c r="D28" s="133"/>
+      <c r="D28" s="101"/>
       <c r="E28" s="65" t="s">
         <v>28</v>
       </c>
@@ -3644,10 +3641,10 @@
       <c r="B30" s="64">
         <v>12</v>
       </c>
-      <c r="C30" s="132" t="s">
+      <c r="C30" s="100" t="s">
         <v>53</v>
       </c>
-      <c r="D30" s="133"/>
+      <c r="D30" s="101"/>
       <c r="E30" s="65" t="s">
         <v>54</v>
       </c>
@@ -3692,8 +3689,8 @@
     <row r="31" spans="1:31" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="24"/>
-      <c r="C31" s="163"/>
-      <c r="D31" s="96"/>
+      <c r="C31" s="118"/>
+      <c r="D31" s="119"/>
       <c r="E31" s="25"/>
       <c r="F31" s="52">
         <f>G31</f>
@@ -3847,57 +3844,57 @@
     </row>
     <row r="34" spans="1:32" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="30"/>
-      <c r="B34" s="159" t="s">
+      <c r="B34" s="114" t="s">
         <v>36</v>
       </c>
-      <c r="C34" s="160"/>
-      <c r="D34" s="160"/>
-      <c r="E34" s="160"/>
-      <c r="F34" s="160"/>
-      <c r="G34" s="160"/>
-      <c r="H34" s="160"/>
-      <c r="I34" s="160"/>
-      <c r="J34" s="160"/>
-      <c r="K34" s="160"/>
-      <c r="L34" s="160"/>
-      <c r="M34" s="160"/>
-      <c r="N34" s="160"/>
-      <c r="O34" s="160"/>
-      <c r="P34" s="160"/>
-      <c r="Q34" s="160"/>
-      <c r="R34" s="160"/>
-      <c r="S34" s="160"/>
-      <c r="T34" s="160"/>
-      <c r="U34" s="160"/>
-      <c r="V34" s="160"/>
-      <c r="W34" s="160"/>
-      <c r="X34" s="160"/>
-      <c r="Y34" s="160"/>
-      <c r="Z34" s="160"/>
-      <c r="AA34" s="161"/>
-      <c r="AB34" s="162"/>
+      <c r="C34" s="115"/>
+      <c r="D34" s="115"/>
+      <c r="E34" s="115"/>
+      <c r="F34" s="115"/>
+      <c r="G34" s="115"/>
+      <c r="H34" s="115"/>
+      <c r="I34" s="115"/>
+      <c r="J34" s="115"/>
+      <c r="K34" s="115"/>
+      <c r="L34" s="115"/>
+      <c r="M34" s="115"/>
+      <c r="N34" s="115"/>
+      <c r="O34" s="115"/>
+      <c r="P34" s="115"/>
+      <c r="Q34" s="115"/>
+      <c r="R34" s="115"/>
+      <c r="S34" s="115"/>
+      <c r="T34" s="115"/>
+      <c r="U34" s="115"/>
+      <c r="V34" s="115"/>
+      <c r="W34" s="115"/>
+      <c r="X34" s="115"/>
+      <c r="Y34" s="115"/>
+      <c r="Z34" s="115"/>
+      <c r="AA34" s="116"/>
+      <c r="AB34" s="117"/>
       <c r="AC34" s="35"/>
       <c r="AD34" s="26"/>
       <c r="AE34" s="1"/>
     </row>
     <row r="35" spans="1:32" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="43"/>
-      <c r="B35" s="164" t="s">
+      <c r="B35" s="120" t="s">
         <v>2</v>
       </c>
-      <c r="C35" s="156" t="s">
+      <c r="C35" s="109" t="s">
         <v>4</v>
       </c>
-      <c r="D35" s="157"/>
-      <c r="E35" s="134" t="s">
+      <c r="D35" s="110"/>
+      <c r="E35" s="122" t="s">
         <v>55</v>
       </c>
-      <c r="F35" s="136" t="s">
+      <c r="F35" s="124" t="s">
         <v>16</v>
       </c>
-      <c r="G35" s="137"/>
-      <c r="H35" s="137"/>
-      <c r="I35" s="138"/>
+      <c r="G35" s="125"/>
+      <c r="H35" s="125"/>
+      <c r="I35" s="112"/>
       <c r="J35" s="45">
         <f>Z19+1</f>
         <v>46097</v>
@@ -3971,10 +3968,10 @@
     </row>
     <row r="36" spans="1:32" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="43"/>
-      <c r="B36" s="165"/>
-      <c r="C36" s="158"/>
-      <c r="D36" s="138"/>
-      <c r="E36" s="135"/>
+      <c r="B36" s="121"/>
+      <c r="C36" s="111"/>
+      <c r="D36" s="112"/>
+      <c r="E36" s="123"/>
       <c r="F36" s="39" t="s">
         <v>56</v>
       </c>
@@ -4063,10 +4060,10 @@
       <c r="B37" s="36">
         <v>1</v>
       </c>
-      <c r="C37" s="102" t="s">
+      <c r="C37" s="130" t="s">
         <v>21</v>
       </c>
-      <c r="D37" s="103"/>
+      <c r="D37" s="105"/>
       <c r="E37" s="21" t="s">
         <v>60</v>
       </c>
@@ -4137,10 +4134,10 @@
       <c r="B38" s="36">
         <v>2</v>
       </c>
-      <c r="C38" s="108" t="s">
+      <c r="C38" s="113" t="s">
         <v>27</v>
       </c>
-      <c r="D38" s="103"/>
+      <c r="D38" s="105"/>
       <c r="E38" s="21" t="s">
         <v>61</v>
       </c>
@@ -4201,10 +4198,10 @@
       <c r="B39" s="36">
         <v>3</v>
       </c>
-      <c r="C39" s="112" t="s">
+      <c r="C39" s="106" t="s">
         <v>31</v>
       </c>
-      <c r="D39" s="103"/>
+      <c r="D39" s="105"/>
       <c r="E39" s="21" t="s">
         <v>62</v>
       </c>
@@ -4275,10 +4272,10 @@
       <c r="B40" s="36">
         <v>5</v>
       </c>
-      <c r="C40" s="112" t="s">
+      <c r="C40" s="106" t="s">
         <v>35</v>
       </c>
-      <c r="D40" s="103"/>
+      <c r="D40" s="105"/>
       <c r="E40" s="21" t="s">
         <v>63</v>
       </c>
@@ -4346,10 +4343,10 @@
       <c r="B41" s="64">
         <v>6</v>
       </c>
-      <c r="C41" s="112" t="s">
+      <c r="C41" s="106" t="s">
         <v>38</v>
       </c>
-      <c r="D41" s="103"/>
+      <c r="D41" s="105"/>
       <c r="E41" s="65" t="s">
         <v>64</v>
       </c>
@@ -4420,10 +4417,10 @@
       <c r="B42" s="64">
         <v>7</v>
       </c>
-      <c r="C42" s="112" t="s">
+      <c r="C42" s="106" t="s">
         <v>41</v>
       </c>
-      <c r="D42" s="103"/>
+      <c r="D42" s="105"/>
       <c r="E42" s="65" t="s">
         <v>42</v>
       </c>
@@ -4494,10 +4491,10 @@
       <c r="B43" s="86">
         <v>9</v>
       </c>
-      <c r="C43" s="153" t="s">
+      <c r="C43" s="104" t="s">
         <v>44</v>
       </c>
-      <c r="D43" s="103"/>
+      <c r="D43" s="105"/>
       <c r="E43" s="65" t="s">
         <v>28</v>
       </c>
@@ -4568,10 +4565,10 @@
       <c r="B44" s="86">
         <v>10</v>
       </c>
-      <c r="C44" s="132" t="s">
+      <c r="C44" s="100" t="s">
         <v>47</v>
       </c>
-      <c r="D44" s="133"/>
+      <c r="D44" s="101"/>
       <c r="E44" s="65" t="s">
         <v>28</v>
       </c>
@@ -4642,10 +4639,10 @@
       <c r="B45" s="88">
         <v>11</v>
       </c>
-      <c r="C45" s="151" t="s">
+      <c r="C45" s="102" t="s">
         <v>49</v>
       </c>
-      <c r="D45" s="152"/>
+      <c r="D45" s="103"/>
       <c r="E45" s="89" t="s">
         <v>65</v>
       </c>
@@ -4716,10 +4713,10 @@
       <c r="B46" s="88">
         <v>12</v>
       </c>
-      <c r="C46" s="132" t="s">
+      <c r="C46" s="100" t="s">
         <v>53</v>
       </c>
-      <c r="D46" s="133"/>
+      <c r="D46" s="101"/>
       <c r="E46" s="89" t="s">
         <v>54</v>
       </c>
@@ -4784,8 +4781,8 @@
     <row r="47" spans="1:32" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
       <c r="B47" s="87"/>
-      <c r="C47" s="129"/>
-      <c r="D47" s="130"/>
+      <c r="C47" s="142"/>
+      <c r="D47" s="143"/>
       <c r="E47" s="37"/>
       <c r="F47" s="55">
         <f t="shared" si="21"/>
@@ -13707,7 +13704,82 @@
       <c r="B991" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="89">
+  <mergeCells count="91">
+    <mergeCell ref="P12:S12"/>
+    <mergeCell ref="P10:S10"/>
+    <mergeCell ref="P9:S9"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="P8:U8"/>
+    <mergeCell ref="P6:S6"/>
+    <mergeCell ref="P7:S7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="P4:S4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="P11:S11"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:D4"/>
+    <mergeCell ref="E3:F4"/>
+    <mergeCell ref="G3:H4"/>
+    <mergeCell ref="E2:L2"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="P3:U3"/>
+    <mergeCell ref="P5:S5"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="P13:S13"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="B18:AB18"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="C43:D43"/>
@@ -13724,79 +13796,6 @@
     <mergeCell ref="E19:E20"/>
     <mergeCell ref="F19:I19"/>
     <mergeCell ref="C27:D27"/>
-    <mergeCell ref="P13:S13"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="B18:AB18"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="P11:S11"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:D4"/>
-    <mergeCell ref="E3:F4"/>
-    <mergeCell ref="G3:H4"/>
-    <mergeCell ref="E2:L2"/>
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="P3:U3"/>
-    <mergeCell ref="P5:S5"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="P4:S4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="P12:S12"/>
-    <mergeCell ref="P10:S10"/>
-    <mergeCell ref="P9:S9"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="P8:U8"/>
-    <mergeCell ref="P6:S6"/>
-    <mergeCell ref="P7:S7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:F8"/>
   </mergeCells>
   <conditionalFormatting sqref="J21:Z29 J30 Y30:Z30">
     <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">

</xml_diff>